<commit_message>
Removing old useless line in medCodeLLM, updates to some results tables
</commit_message>
<xml_diff>
--- a/resultsOrgRecDiff.xlsx
+++ b/resultsOrgRecDiff.xlsx
@@ -462,10 +462,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.4846938775510204</v>
+        <v>0.06152549515381374</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5153061224489797</v>
+        <v>0.9384745048461862</v>
       </c>
     </row>
     <row r="3">
@@ -480,28 +480,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9792566983578219</v>
+        <v>0.9798918918918919</v>
       </c>
       <c r="D3" t="n">
-        <v>0.02074330164217808</v>
+        <v>0.02010810810810815</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>gemma3:4b</t>
+          <t>gpt-oss:20b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>doctorNotes/note4.txt</t>
+          <t>Model Failed JSON gen</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.8986928104575164</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1013071895424836</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -516,10 +516,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.9811647542758173</v>
+        <v>0.9796712802768166</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01883524572418271</v>
+        <v>0.0203287197231834</v>
       </c>
     </row>
     <row r="6">
@@ -534,10 +534,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9744920017293558</v>
+        <v>0.9794683380159931</v>
       </c>
       <c r="D6" t="n">
-        <v>0.02550799827064421</v>
+        <v>0.02053166198400691</v>
       </c>
     </row>
     <row r="7">
@@ -552,10 +552,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.05765199161425576</v>
+        <v>0.9379785604900459</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9423480083857443</v>
+        <v>0.06202143950995409</v>
       </c>
     </row>
     <row r="8">
@@ -570,28 +570,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.9689719626168224</v>
+        <v>0.06531204644412192</v>
       </c>
       <c r="D8" t="n">
-        <v>0.03102803738317761</v>
+        <v>0.9346879535558781</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>gemma3:4b</t>
+          <t>gpt-oss:20b</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>doctorNotes/note5.txt</t>
+          <t>Model Failed JSON gen</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.8998435054773083</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1001564945226917</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -606,10 +606,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.9617242660720922</v>
+        <v>0.9639271104499814</v>
       </c>
       <c r="D10" t="n">
-        <v>0.03827573392790784</v>
+        <v>0.03607288955001864</v>
       </c>
     </row>
     <row r="11">
@@ -624,10 +624,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.9624953583364277</v>
+        <v>0.9628804751299184</v>
       </c>
       <c r="D11" t="n">
-        <v>0.03750464166357226</v>
+        <v>0.03711952487008163</v>
       </c>
     </row>
     <row r="12">
@@ -642,10 +642,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.6355296080066722</v>
+        <v>0.5311820159535896</v>
       </c>
       <c r="D12" t="n">
-        <v>0.3644703919933278</v>
+        <v>0.4688179840464104</v>
       </c>
     </row>
     <row r="13">
@@ -660,28 +660,28 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.9582974535613237</v>
+        <v>0.9697422487859544</v>
       </c>
       <c r="D13" t="n">
-        <v>0.04170254643867632</v>
+        <v>0.03025775121404561</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>gemma3:4b</t>
+          <t>gpt-oss:20b</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>doctorNotes/note1.txt</t>
+          <t>Model Failed JSON gen</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.8892468787756745</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1107531212243255</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -696,10 +696,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.07151314231588918</v>
+        <v>0.960840024706609</v>
       </c>
       <c r="D15" t="n">
-        <v>0.9284868576841108</v>
+        <v>0.03915997529339099</v>
       </c>
     </row>
     <row r="16">
@@ -714,10 +714,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.9749624436654982</v>
+        <v>0.9698855151816824</v>
       </c>
       <c r="D16" t="n">
-        <v>0.02503755633450178</v>
+        <v>0.03011448481831758</v>
       </c>
     </row>
     <row r="17">
@@ -732,10 +732,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.9746646795827124</v>
+        <v>0.452801805189921</v>
       </c>
       <c r="D17" t="n">
-        <v>0.02533532041728759</v>
+        <v>0.547198194810079</v>
       </c>
     </row>
     <row r="18">
@@ -750,28 +750,28 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.9799899949974987</v>
+        <v>0.97530556248441</v>
       </c>
       <c r="D18" t="n">
-        <v>0.02001000500250127</v>
+        <v>0.02469443751558997</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>gemma3:4b</t>
+          <t>gpt-oss:20b</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>doctorNotes/note2.txt</t>
+          <t>Model Failed JSON gen</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.9690464303544682</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>0.03095356964553175</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -786,10 +786,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.9717599596570852</v>
+        <v>0.9824824824824825</v>
       </c>
       <c r="D20" t="n">
-        <v>0.02824004034291483</v>
+        <v>0.01751751751751751</v>
       </c>
     </row>
     <row r="21">
@@ -804,10 +804,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.976083707025411</v>
+        <v>0.9810094952523738</v>
       </c>
       <c r="D21" t="n">
-        <v>0.02391629297458897</v>
+        <v>0.0189905047476262</v>
       </c>
     </row>
     <row r="22">
@@ -822,10 +822,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.6842780200051295</v>
+        <v>0.4448529411764706</v>
       </c>
       <c r="D22" t="n">
-        <v>0.3157219799948705</v>
+        <v>0.5551470588235294</v>
       </c>
     </row>
     <row r="23">
@@ -840,28 +840,28 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.9713275726630007</v>
+        <v>0.956964006259781</v>
       </c>
       <c r="D23" t="n">
-        <v>0.02867242733699926</v>
+        <v>0.04303599374021905</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>gemma3:4b</t>
+          <t>gpt-oss:20b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>doctorNotes/note3.txt</t>
+          <t>Model Failed JSON gen</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.963749248948528</v>
+        <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>0.03625075105147202</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -876,10 +876,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.9680705190989226</v>
+        <v>0.9728880157170924</v>
       </c>
       <c r="D25" t="n">
-        <v>0.03192948090107739</v>
+        <v>0.02711198428290762</v>
       </c>
     </row>
     <row r="26">
@@ -894,10 +894,10 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.9673998428908092</v>
+        <v>0.9749216300940439</v>
       </c>
       <c r="D26" t="n">
-        <v>0.03260015710919084</v>
+        <v>0.02507836990595613</v>
       </c>
     </row>
   </sheetData>

</xml_diff>